<commit_message>
Phase 2 complete: full source collection across sections 2.1-2.11 (market sizing, Germany deep dive, Amazon competitor analysis, category analysis, longevity deep dive, brand analysis, review mining, product formats, pricing, keyword research, regulatory overview)
</commit_message>
<xml_diff>
--- a/01_Screenshots_and_Sources/Data_Source_Documentation.xlsx
+++ b/01_Screenshots_and_Sources/Data_Source_Documentation.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sai/Desktop/Upwork Projects/Amazon Market Research - European Dog Supplements/01_Screenshots_and_Sources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sai/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41DDE196-77FF-FE45-AA03-3247C868F662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0042CF10-5BAB-AD4D-9DAD-318CA0D7EDAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="18440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Source Log" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="386">
   <si>
     <t>Fact ID</t>
   </si>
@@ -812,13 +812,379 @@
   </si>
   <si>
     <t>Example of a human-wellness/longevity brand extending into pet - directly analogous positioning to the client's own proposed brand concept (human-longevity-adjacent brand entering pet space)</t>
+  </si>
+  <si>
+    <t>MKT-042</t>
+  </si>
+  <si>
+    <t>Review Mining - Palatability</t>
+  </si>
+  <si>
+    <t>Recurring theme across German and English-language review sources: dogs refusing to eat/take supplements is one of the most common complaints, especially for tablet/capsule formats without a strong flavor. German source explicitly notes tablet forms have 'kein fleischiger Geschmack' (no meaty flavor dogs love), making administration harder; sources recommend powder/oil formats or flavored (beef/liver) tablets specifically to counter this</t>
+  </si>
+  <si>
+    <t>Haustier Bewertungen; Vergleich.org; PETBOOK</t>
+  </si>
+  <si>
+    <t>https://www.haustierbewertungen.de/die-wahrheit-uber-hunde-nahrungserganzungsmittel-fur-gelenke.php ; https://www.vergleich.org/hunde-ergaenzungsfutter/</t>
+  </si>
+  <si>
+    <t>Verified (cross-referenced, consistent across German sources)</t>
+  </si>
+  <si>
+    <t>MKT-043</t>
+  </si>
+  <si>
+    <t>Review Mining - Efficacy Skepticism</t>
+  </si>
+  <si>
+    <t>Very common review pattern (English-language, Chewy/Walmart): customers report 'no noticeable difference' after 1-2 containers and cancel subscriptions; one reviewer explicitly credits marketing/advertising for the initial purchase decision but rates only 3 stars due to inconclusive results. This reflects a structural challenge: joint/mobility benefits take 4-6 weeks minimum to show (per MedicAnimal), longer than many buyers' patience or single-purchase window</t>
+  </si>
+  <si>
+    <t>Chewy.com customer reviews (WINPRO PET); MedicAnimal</t>
+  </si>
+  <si>
+    <t>https://www.chewy.com/winpro-pet-hip-joint-soft-chews-dog/product-reviews/199709 ; https://medicanimal.com/blogs/pet-advice/do-joint-supplements-work-for-dogs-a-complete-guide</t>
+  </si>
+  <si>
+    <t>Verified (direct customer review quotes)</t>
+  </si>
+  <si>
+    <t>MKT-044</t>
+  </si>
+  <si>
+    <t>Review Mining - GI Side Effects</t>
+  </si>
+  <si>
+    <t>Mild digestive upset (loose stools, vomiting, gas) is a recurring but generally minor complaint across joint supplements specifically, most commonly associated with glucosamine at high doses or turmeric without an absorption aid (e.g. black pepper/piperine). Sources are consistent that these effects are typically mild and often resolve within days, but they still show up repeatedly as a source of buyer anxiety/complaint in reviews</t>
+  </si>
+  <si>
+    <t>PetMD; Pet Honesty; Simon Vet Surgical; Walmart customer reviews; MedicAnimal</t>
+  </si>
+  <si>
+    <t>https://www.petmd.com/dog/nutrition/glucosamine-for-dogs ; https://www.pethonesty.com/blogs/blog/best-joint-supplement-for-dogs ; https://www.simonvetsurgical.com/news/the-top-10-supplements-for-dogs-with-arthritis</t>
+  </si>
+  <si>
+    <t>Verified (cross-referenced across 5 sources)</t>
+  </si>
+  <si>
+    <t>MKT-045</t>
+  </si>
+  <si>
+    <t>Review Mining - Packaging Complaints</t>
+  </si>
+  <si>
+    <t>Specific, concrete packaging complaints found in reviews: soft chews sticking together in the container (freshness/storage issue); peel-off backing on topical/patch-style products being difficult to remove and leaving residue; oil bottles leaking when tipped over; instructions/dosing text printed too small to read without a phone camera to zoom in</t>
+  </si>
+  <si>
+    <t>Walmart.com customer reviews; Hundeshop.de reviews</t>
+  </si>
+  <si>
+    <t>https://www.walmart.com/reviews/product/5719756457 ; https://www.hundeshop.de/hund/ernaehrung/nahrungsergaenzung/bewertungen/</t>
+  </si>
+  <si>
+    <t>Direct, specific packaging pain points - concrete and actionable for product design</t>
+  </si>
+  <si>
+    <t>MKT-046</t>
+  </si>
+  <si>
+    <t>Review Mining - Ingredient/Trust Concerns</t>
+  </si>
+  <si>
+    <t>Independent lab testing (ConsumerLab.com, cited by NBC News) found 4 of 6 tested joint supplements for pets failed to meet their labeled glucosamine/chondroitin content or had other quality flaws, including lead contamination in some cases; a wider trade-group test of 87 brands found roughly one-quarter fell short of label claims. OTC pet supplements face substantially less regulatory scrutiny than human supplements or pet drugs</t>
+  </si>
+  <si>
+    <t>NBC News (reporting on ConsumerLab.com testing)</t>
+  </si>
+  <si>
+    <t>https://www.nbcnews.com/health/health-news/many-pet-supplements-don-t-meet-claims-flna1C9450237</t>
+  </si>
+  <si>
+    <t>Verified (independent lab testing, reported by a major news outlet)</t>
+  </si>
+  <si>
+    <t>Significant trust-gap finding: label accuracy/quality verification (e.g. third-party testing, COAs) is a credible, provable differentiator, not just a marketing claim - directly usable as a genuine USP</t>
+  </si>
+  <si>
+    <t>MKT-047</t>
+  </si>
+  <si>
+    <t>Review Mining - Positive Sentiment / Repeat Purchase Drivers</t>
+  </si>
+  <si>
+    <t>Positive reviews (Zooplus UK, German retailer reviews) consistently cite: visible mobility improvement (dog running/playing again without discomfort), ease of administration when disguised in food/treat, and long-term consistent use correlating with sustained results. Repeat purchase appears strongly tied to the dog owner personally observing a behavioral change (e.g., 'racing around at high speed with no discomfort'), not to abstract label claims</t>
+  </si>
+  <si>
+    <t>Zooplus.com/feedback (LUPOSAN reviews); Hundeshop.de</t>
+  </si>
+  <si>
+    <t>https://zooplus.com/feedback/shop/dogs/supplements_specialty_food/bones_joints/luposan/129094 ; https://www.hundeshop.de/hund/ernaehrung/nahrungsergaenzung/bewertungen/</t>
+  </si>
+  <si>
+    <t>MKT-048</t>
+  </si>
+  <si>
+    <t>Product Formats - Global Share</t>
+  </si>
+  <si>
+    <t>Soft chews/chewables hold the largest global format share: estimates range 43.84% (Fortune Business Insights, 2026), 46%+ (Woodstone Research, 2025), and 47.6% specifically within private-label (Future Market Insights, 2026). Tablets &amp; capsules are consistently the second-largest global format. All sources agree chews dominate due to palatability, ease of administration, and perceived effectiveness</t>
+  </si>
+  <si>
+    <t>Fortune Business Insights; Woodstone Research; Future Market Insights</t>
+  </si>
+  <si>
+    <t>https://www.fortunebusinessinsights.com/pet-supplements-market-109797 ; https://www.woodstoneresearch.com/reports/pet-dietary-supplements-market ; https://www.futuremarketinsights.com/reports/private-label-pet-supplement-market</t>
+  </si>
+  <si>
+    <t>Estimate (cross-referenced across 3 independent market research firms, consistent direction and magnitude)</t>
+  </si>
+  <si>
+    <t>MKT-049</t>
+  </si>
+  <si>
+    <t>Product Formats - Growth by Format</t>
+  </si>
+  <si>
+    <t>Powders are the fastest-growing format specifically, at 11.2% CAGR through 2031 (Mordor Intelligence), driven by compatibility with personalized/algorithmic dosing and lower per-unit manufacturing cost. Liquids/gels are also cited as a strong-growth format (Precedence Research) as manufacturers move 'beyond traditional tablets and powders' - e.g. Pet Honesty launched a new liquid format across hip/joint, skin/coat, and multivitamin lines in August 2024</t>
+  </si>
+  <si>
+    <t>Mordor Intelligence; Precedence Research; Woodstone Research</t>
+  </si>
+  <si>
+    <t>https://www.mordorintelligence.com/industry-reports/pet-dietary-supplements-market ; https://www.precedenceresearch.com/pet-dietary-supplements-market ; https://www.woodstoneresearch.com/reports/pet-dietary-supplements-market</t>
+  </si>
+  <si>
+    <t>Estimate (cross-referenced, consistent)</t>
+  </si>
+  <si>
+    <t>Important nuance: chews dominate on CURRENT share, but powders and liquids are growing fastest - a new entrant isn't purely locked into copying the leading format</t>
+  </si>
+  <si>
+    <t>MKT-050</t>
+  </si>
+  <si>
+    <t>Product Formats - EU Regulatory Note (Chews)</t>
+  </si>
+  <si>
+    <t>The European Food Safety Authority (EFSA) has raised concerns about certain gelling agents used in soft chews, prompting manufacturers to reformulate with EFSA-approved alternatives such as carrageenan and agar</t>
+  </si>
+  <si>
+    <t>Mordor Intelligence (Pet Dietary Supplements Market)</t>
+  </si>
+  <si>
+    <t>Estimate (single source - flagged for verification, not independently corroborated in this pass)</t>
+  </si>
+  <si>
+    <t>Directly relevant if the new brand chooses a soft-chew format for EU sale - gelling agent selection needs to be EFSA-compliant from formulation stage, not retrofitted later. Single-source claim - worth confirming with a formulation/regulatory specialist before treating as settled</t>
+  </si>
+  <si>
+    <t>MKT-051</t>
+  </si>
+  <si>
+    <t>Pricing - mammaly (Amazon Marketplace/Fressnapf)</t>
+  </si>
+  <si>
+    <t>mammaly product pricing observed: Happy HIPS joint treats (110g, ~30 snacks) EUR17.99-19.95 (base price ~EUR0.60/piece); 15-in-1 Multivitamin Complex (110g, 30 treats) EUR19.95 (EUR181.36/kg); Fresh Smile dental (110g) EUR16.99 (EUR154.45/kg) at Fressnapf. mammaly won 1st place at the Fressnapf Innovation Award (2022). A customer review explicitly states they switched away from mammaly's Happy HIPS to a competitor because mammaly's price had increased ('der Preis so erhöht')</t>
+  </si>
+  <si>
+    <t>futter-und-tierbedarf.de; Amazon.de customer reviews; Fressnapf.de</t>
+  </si>
+  <si>
+    <t>https://www.futter-und-tierbedarf.de/Hunde/Hundefutter/Hundefutter-von-mammaly/Preis-25 ; https://www.amazon.de/Gelenktabletten-Gr%C3%BCnlippmuschel-Hund-mammaly-Knorpelroduktion/dp/B0DJL9RLGP</t>
+  </si>
+  <si>
+    <t>Verified (live retailer listings + direct customer review quote)</t>
+  </si>
+  <si>
+    <t>Direct evidence that mammaly's core price point sits around EUR17-20 per 110g pack, and that customers ARE price-sensitive enough to switch brands over increases - useful ceiling/elasticity signal for premium positioning</t>
+  </si>
+  <si>
+    <t>MKT-052</t>
+  </si>
+  <si>
+    <t>Pricing - Fressnapf Marketplace Joint Tablets (mid-market cluster)</t>
+  </si>
+  <si>
+    <t>Multiple mid-market joint tablet brands found on Fressnapf's online marketplace, all German-made, similar green-lipped-mussel/MSM/devil's claw formulas, positioned as accessible alternatives to premium DTC brands: Wolfsbacher Natur (365 tablets), BeG Buddy (150g, 100 tablets/~6 months supply), Pfotenkumpels Hüftschwung (200g), Annimally (120 tablets). Exact prices not captured in this pass (Fressnapf's marketplace prices require login/session-specific rendering), but positioning language ('günstige Preise', value multi-packs) signals a mid-market tier below premium DTC pricing</t>
+  </si>
+  <si>
+    <t>Fressnapf.de product listings (Wolfsbacher, BeG Buddy, Pfotenkumpels, Annimally)</t>
+  </si>
+  <si>
+    <t>https://www.fressnapf.de/p/wolfsbacher-natur-gelenktabletten-365-stueck-1678079/ ; https://www.fressnapf.de/p/beg-buddy-gelenktabletten-hund-gruenlippmuschel-gelenk-hund-150g-1457251/ ; https://www.fressnapf.de/p/annimally-gelenktabletten-120-stueck-1721723/</t>
+  </si>
+  <si>
+    <t>Verified (product existence and formulation) / Estimate (pricing tier, exact price not captured)</t>
+  </si>
+  <si>
+    <t>Confirms a crowded mid-market tier of near-identical German 'natural joint tablet' formulas exists between mass-market (8in1-style) and premium DTC (mammaly/YuMOVE) pricing - exact price points flagged as a gap for a dedicated Amazon/Fressnapf pricing tool pull</t>
+  </si>
+  <si>
+    <t>MKT-053</t>
+  </si>
+  <si>
+    <t>IMPORTANT CORRECTION to MKT-030</t>
+  </si>
+  <si>
+    <t>mammaly (the client's closest direct competitor, per MKT-017) already operates a dedicated 'Langlebigkeit' (Longevity) product collection on its own German-language website, including a 'Long Life Zellpower' antioxidant snack product explicitly marketed to 'protect cells and slow the aging process' (Zellen schützen, Alterungsprozess verlangsamen). This means the Section 2.4/2.5 finding of 'zero longevity competition in Germany' was accurate specifically for Amazon.de search results, but is NOT accurate for the German market as a whole once DTC brand websites are included</t>
+  </si>
+  <si>
+    <t>mammaly.de official collection page</t>
+  </si>
+  <si>
+    <t>https://www.mammaly.de/collections/langlebigkeit</t>
+  </si>
+  <si>
+    <t>Verified (brand's own live site)</t>
+  </si>
+  <si>
+    <t>CRITICAL CORRECTION - revises MKT-030 and the Section 2.5 opportunity assessment. The white space is narrower than first identified: it is specifically 'science-forward, NMN/NAD+-style longevity supplements on Amazon.de,' not 'longevity products in the German market' broadly. mammaly has already claimed the general 'Langlebigkeit' consumer positioning and German-language search terms with an antioxidant-based (not NMN-based) formulation - directly relevant competitive intelligence the client needs before finalizing a longevity product strategy</t>
+  </si>
+  <si>
+    <t>MKT-054</t>
+  </si>
+  <si>
+    <t>Keyword Demand - German Longevity/Anti-Aging Content</t>
+  </si>
+  <si>
+    <t>Multiple independent German-language editorial/vet sources actively publish content using the terms 'Langlebigkeit' (longevity), 'Gesundes Altern' (healthy aging), and 'Anti-Aging Hund' in dog-health contexts (e.g. 'Longevity für Hunde: Fit und gesund bis ins hohe Alter', '20 Anti-Aging Tipps für Hunde'), referencing concepts like caloric restriction extending lifespan by up to 1.8 years, sarcopenia (muscle loss) prevention, and cognitive dysfunction. This indicates the underlying consumer/content-side vocabulary and interest already exists in German, independent of any specific product</t>
+  </si>
+  <si>
+    <t>Herz für Tiere; Bugbell.de; Purapep.de; Dr. Hölter Tierarzt</t>
+  </si>
+  <si>
+    <t>https://herz-fuer-tiere.de/haustiere/hunde/gesundheit-und-vorsorge-bei-hunden/longevity-fuer-hunde ; https://bugbell.de/blogs/news/20-dinge-die-das-leben-deines-hundes-verlangern ; https://www.purapep.de/ratgeber/hundeleben/ernaehrung-hund-im-alter/</t>
+  </si>
+  <si>
+    <t>Verified (multiple independent editorial sources)</t>
+  </si>
+  <si>
+    <t>Reinforces that 'Langlebigkeit'/'gesundes Altern' is a real, actively-used German search/content vocabulary - supports treating longevity as a genuine (if now partially contested) opportunity rather than a concept with no German-language footing at all</t>
+  </si>
+  <si>
+    <t>MKT-055</t>
+  </si>
+  <si>
+    <t>Keyword Demand - Joint Category (search-trend cross-check)</t>
+  </si>
+  <si>
+    <t>Cross-referencing MKT-021: the 'Gelenktabletten Hund' niche shows +6.2% 90-day search growth per Flapen, and independent listings on eBay.de and comparison sites (HundeINFOPortal) confirm sustained purchase volume ('134 Personen haben dieses Produkt kürzlich gekauft' / 'mehr als 10 verfügbar, 42 verkauft'). At least 15 comparison-tested products exist in German-language 'Gelenktabletten Hunde' buying-guide content specifically (HundeINFOPortal), confirming this is an actively searched, high-content-volume category in German, not just an English-language pattern</t>
+  </si>
+  <si>
+    <t>Flapen; HundeINFOPortal; eBay.de listings</t>
+  </si>
+  <si>
+    <t>https://flapen.com/research/de/haustier/gelenktabletten-hund ; https://www.hundeinfoportal.de/ratgeber/futter-ratgeber/hundefutter/nahrungsergaenzungen-vitamine-fuer-hunde/gelenktabletten/ ; https://www.ebay.de/itm/316869448922</t>
+  </si>
+  <si>
+    <t>Verified (cross-referenced across 3 independent sources)</t>
+  </si>
+  <si>
+    <t>MKT-056</t>
+  </si>
+  <si>
+    <t>Regulatory - Feed Classification</t>
+  </si>
+  <si>
+    <t>Under EU feed law (Regulation (EC) 767/2009) and the German LFGB (Lebensmittel- und Futtermittelgesetzbuch), a dog supplement must be labeled as either an 'Alleinfuttermittel' (complete feed - mathematically covers full daily nutrient needs) or an 'Ergänzungsfuttermittel' (complementary/supplementary feed - does not cover full nutrient needs alone and must be combined with other feed). Nearly all dog supplements (vitamins, joint support, probiotics, etc.) fall under 'Ergänzungsfuttermittel.' This is a mandatory on-label declaration, not optional marketing language</t>
+  </si>
+  <si>
+    <t>Petman.de; Haendlerbund.de; Fresstipp.de</t>
+  </si>
+  <si>
+    <t>https://petman.de/ueber-barf/futtermittelrecht-deklarationen/alleinfuttermittel ; https://www.haendlerbund.de/de/ratgeber/branchen/3748-tierfutter-verordnung ; https://fresstipp.de/deklaration-von-hunde-und-katzenfutter/</t>
+  </si>
+  <si>
+    <t>Verified (cross-referenced across 3 independent legal/industry sources)</t>
+  </si>
+  <si>
+    <t>MKT-057</t>
+  </si>
+  <si>
+    <t>Regulatory - Business Registration</t>
+  </si>
+  <si>
+    <t>Feed business operators (including online sellers) placing feed on the market in Germany/EU must register with the competent authority (in Germany, coordinated via the BVL - Bundesamt für Verbraucherschutz und Lebensmittelsicherheit) under Regulation (EC) 183/2005 (feed hygiene) and Article 9/Article 5(2) requirements, and must implement a HACCP-based food/feed safety system. This applies to the responsible labeling entity, not just the physical manufacturer, if they are different parties (relevant for a brand using contract/private-label manufacturing)</t>
+  </si>
+  <si>
+    <t>BVL official guidance documents (Leitfaden zur Registrierung von Futtermittelunternehmen; FAQ for online feed trade)</t>
+  </si>
+  <si>
+    <t>https://www.bvl.bund.de/SharedDocs/Downloads/02_Futtermittel/fm_Leitfaden_Registrierung_Betriebe.pdf ; https://www.bvl.bund.de/SharedDocs/Downloads/03_Verbraucherprodukte/FAQ/FAQ_Futtermittelunternehmen_Online-Handel.pdf</t>
+  </si>
+  <si>
+    <t>Verified (official German government source)</t>
+  </si>
+  <si>
+    <t>Directly actionable: if the client's brand uses a contract manufacturer but handles its own labeling/branding, IT (not just the manufacturer) likely needs its own BVL registration as the 'kennzeichnungsverantwortlicher Inverkehrbringer' (labeling-responsible market-placer) - a concrete compliance step to plan for, not just the manufacturer's responsibility alone</t>
+  </si>
+  <si>
+    <t>MKT-058</t>
+  </si>
+  <si>
+    <t>Regulatory - Mandatory Labeling Elements</t>
+  </si>
+  <si>
+    <t>Mandatory label elements for a German/EU dog supplement include: feed type designation (Ergänzungsfuttermittel), target species/category, net weight/volume, name and address of the labeling-responsible feed business operator, the operator's registration/approval number (if the labeling party is not the manufacturer), full list of individual feed materials/ingredients, all additives with name/E-number, group designation (e.g. nutritional additive, technological additive, sensory additive) and quantity added, and prescribed analytical constituents per EU Annexes VI/VII. Moisture content must be declared if above 14%</t>
+  </si>
+  <si>
+    <t>BVL FAQ (Online-Handel); Napfcheck.de; FEDIAF Kodex für gute Kennzeichnung von Heimtierfuttermitteln</t>
+  </si>
+  <si>
+    <t>https://www.bvl.bund.de/SharedDocs/Downloads/03_Verbraucherprodukte/FAQ/FAQ_Futtermittelunternehmen_Online-Handel.pdf ; https://www.napfcheck.de/deklaration-was-gehoert-aufs-etikett/ ; https://www.ivh-online.de/fileadmin/ivh/user_upload/Branchenleitlinien/FEDIAF_Kennzeichnung_von_Heimtierfuttermitteln_Okt18.pdf</t>
+  </si>
+  <si>
+    <t>Verified (official government + industry association sources)</t>
+  </si>
+  <si>
+    <t>This is a detailed, actionable label-compliance checklist directly usable for the client's packaging development</t>
+  </si>
+  <si>
+    <t>MKT-059</t>
+  </si>
+  <si>
+    <t>Regulatory - Health Claims</t>
+  </si>
+  <si>
+    <t>Confirmed via MKT-035 and general EU food supplement regulation: functional health claims are tightly restricted - only specific, pre-approved risk-reduction/functional claims are permitted, and general disease-cure/prevention language is prohibited. This applies to both packaging (on-pack) and off-pack marketing materials (website, ads, social media, POS material) per the FEDIAF labeling code definition of regulated communications</t>
+  </si>
+  <si>
+    <t>FEDIAF Kodex für gute Kennzeichnung von Heimtierfuttermitteln; juravendis.de (Futtermittelrecht legal overview)</t>
+  </si>
+  <si>
+    <t>https://www.ivh-online.de/fileadmin/ivh/user_upload/Branchenleitlinien/FEDIAF_Kennzeichnung_von_Heimtierfuttermitteln_Okt18.pdf ; https://www.juravendis.de/healthcare/futtermittelrecht/</t>
+  </si>
+  <si>
+    <t>Important scope note: health-claim restrictions apply to ALL marketing communications, not just the physical label - directly relevant to how the client's future website/Amazon listing copy and social media content must be written, not just packaging</t>
+  </si>
+  <si>
+    <t>MKT-060</t>
+  </si>
+  <si>
+    <t>Regulatory - 'Made in Germany' Signal</t>
+  </si>
+  <si>
+    <t>'Made in Germany' / 'Hergestellt in Deutschland' appears as an explicit trust/marketing claim across numerous competitor products reviewed in this research (Wolfsbacher, BeG Buddy, Pfotenkumpels, dog1, NatiVivo, Veddelholzer) and in listing titles optimized specifically around this phrase (Section 2.10, MKT-055). While the specific legal threshold for using 'Made in Germany' on a feed product was not independently verified with a precise legal citation in this pass, its ubiquity across competitor listings confirms it functions as a significant, actively-used consumer trust signal in this category</t>
+  </si>
+  <si>
+    <t>Multiple competitor listings (Fressnapf, Amazon.de, eBay.de) reviewed across Sections 2.3, 2.6, 2.10</t>
+  </si>
+  <si>
+    <t>See MKT-021, MKT-022, MKT-055 for underlying listings</t>
+  </si>
+  <si>
+    <t>Verified (pattern observed across many listings) / Not independently verified (the precise legal origin-labeling threshold itself)</t>
+  </si>
+  <si>
+    <t>Flagged gap: the exact legal criteria for claiming 'Made in Germany' on a feed product (e.g. required % of manufacturing/formulation occurring in Germany) was not confirmed with a specific regulatory citation in this pass - recommend verifying with a customs/trade-law specialist before using the claim, even though it is clearly commercially valuable</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -838,12 +1204,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -859,7 +1219,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -867,23 +1227,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1187,7 +1556,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1201,1083 +1570,1563 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:8" ht="42" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="4" t="s">
+      <c r="F2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:8" ht="56" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="4" t="s">
+      <c r="F3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:8" ht="56" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="4" t="s">
+      <c r="F4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:8" ht="70" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="4" t="s">
+      <c r="F5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:8" ht="56" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="4" t="s">
+      <c r="F6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:8" ht="42" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="4" t="s">
+      <c r="F7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H7" s="4"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" ht="42" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="4" t="s">
+      <c r="F8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:8" ht="56" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="4" t="s">
+      <c r="F9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="4"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" ht="42" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="F10" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="4" t="s">
+      <c r="F10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:8" ht="56" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F11" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="4" t="s">
+      <c r="F11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="H11" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:8" ht="56" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F12" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="4" t="s">
+      <c r="F12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:8" ht="70" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F13" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="4" t="s">
+      <c r="F13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="H13" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:8" ht="56" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="4" t="s">
+      <c r="F14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H14" s="4"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="4" t="s">
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:8" ht="98" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="F15" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="4" t="s">
+      <c r="F15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="H15" s="4" t="s">
+      <c r="H15" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
+    <row r="16" spans="1:8" ht="70" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F16" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="4" t="s">
+      <c r="F16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="4" t="s">
+    <row r="17" spans="1:8" ht="98" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="F17" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="4" t="s">
+      <c r="F17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="H17" s="2" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="4" t="s">
+    <row r="18" spans="1:8" ht="84" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="F18" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="4" t="s">
+      <c r="F18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="H18" s="2" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
+    <row r="19" spans="1:8" ht="56" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="F19" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" s="4" t="s">
+      <c r="F19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="H19" s="2" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="4" t="s">
+    <row r="20" spans="1:8" ht="70" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="F20" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="4" t="s">
+      <c r="F20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="H20" s="4" t="s">
+      <c r="H20" s="2" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="4" t="s">
+    <row r="21" spans="1:8" ht="140" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="F21" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="4" t="s">
+      <c r="F21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="H21" s="4" t="s">
+      <c r="H21" s="2" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="4" t="s">
+    <row r="22" spans="1:8" ht="84" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="F22" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="4" t="s">
+      <c r="F22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="H22" s="2" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="4" t="s">
+    <row r="23" spans="1:8" ht="140" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="F23" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" s="4" t="s">
+      <c r="F23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="H23" s="4"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="4" t="s">
+      <c r="H23" s="2"/>
+    </row>
+    <row r="24" spans="1:8" ht="42" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="F24" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" s="4" t="s">
+      <c r="F24" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H24" s="4" t="s">
+      <c r="H24" s="2" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="4" t="s">
+    <row r="25" spans="1:8" ht="56" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="F25" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="4" t="s">
+      <c r="F25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H25" s="4" t="s">
+      <c r="H25" s="2" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="4" t="s">
+    <row r="26" spans="1:8" ht="84" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="F26" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" s="4" t="s">
+      <c r="F26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="H26" s="2" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A27" s="4" t="s">
+    <row r="27" spans="1:8" ht="70" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="F27" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" s="4" t="s">
+      <c r="F27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="H27" s="4"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
+      <c r="H27" s="2"/>
+    </row>
+    <row r="28" spans="1:8" ht="70" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="F28" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="4" t="s">
+      <c r="F28" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="H28" s="4"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" s="4" t="s">
+      <c r="H28" s="2"/>
+    </row>
+    <row r="29" spans="1:8" ht="56" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="F29" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G29" s="4" t="s">
+      <c r="F29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H29" s="4" t="s">
+      <c r="H29" s="2" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" s="4" t="s">
+    <row r="30" spans="1:8" ht="98" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="F30" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="4" t="s">
+      <c r="F30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="H30" s="4" t="s">
+      <c r="H30" s="2" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" s="4" t="s">
+    <row r="31" spans="1:8" ht="84" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="E31" s="4" t="s">
+      <c r="E31" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="F31" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G31" s="4" t="s">
+      <c r="F31" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="H31" s="4" t="s">
+      <c r="H31" s="2" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="4" t="s">
+    <row r="32" spans="1:8" ht="84" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="D32" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="E32" s="4" t="s">
+      <c r="E32" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="F32" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" s="4" t="s">
+      <c r="F32" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="H32" s="4" t="s">
+      <c r="H32" s="2" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="4" t="s">
+    <row r="33" spans="1:8" ht="84" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D33" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="E33" s="4" t="s">
+      <c r="E33" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="F33" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G33" s="4" t="s">
+      <c r="F33" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G33" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="H33" s="4" t="s">
+      <c r="H33" s="2" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" s="4" t="s">
+    <row r="34" spans="1:8" ht="140" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D34" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="E34" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="F34" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G34" s="4" t="s">
+      <c r="F34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G34" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="H34" s="4" t="s">
+      <c r="H34" s="2" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" s="4" t="s">
+    <row r="35" spans="1:8" ht="154" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="D35" s="4" t="s">
+      <c r="D35" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="E35" s="4" t="s">
+      <c r="E35" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="F35" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G35" s="4" t="s">
+      <c r="F35" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G35" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="H35" s="4" t="s">
+      <c r="H35" s="2" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" s="4" t="s">
+    <row r="36" spans="1:8" ht="112" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C36" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="D36" s="4" t="s">
+      <c r="D36" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="E36" s="4" t="s">
+      <c r="E36" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="F36" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G36" s="4" t="s">
+      <c r="F36" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G36" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="H36" s="4" t="s">
+      <c r="H36" s="2" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37" s="4" t="s">
+    <row r="37" spans="1:8" ht="84" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C37" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="D37" s="4" t="s">
+      <c r="D37" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="E37" s="4" t="s">
+      <c r="E37" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="F37" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G37" s="4" t="s">
+      <c r="F37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G37" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H37" s="4" t="s">
+      <c r="H37" s="2" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A38" s="1" t="s">
+    <row r="38" spans="1:8" ht="98" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C38" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D38" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="E38" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="F38" s="2">
-        <v>46249</v>
-      </c>
-      <c r="G38" s="1" t="s">
+      <c r="F38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G38" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="H38" s="1" t="s">
+      <c r="H38" s="2" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A39" s="1" t="s">
+    <row r="39" spans="1:8" ht="70" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C39" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="D39" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="E39" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="F39" s="2">
-        <v>46249</v>
-      </c>
-      <c r="G39" s="1" t="s">
+      <c r="F39" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G39" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H39" s="1" t="s">
+      <c r="H39" s="2" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" s="1" t="s">
+    <row r="40" spans="1:8" ht="84" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D40" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="E40" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="F40" s="2">
-        <v>46249</v>
-      </c>
-      <c r="G40" s="1" t="s">
+      <c r="F40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G40" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="H40" s="1" t="s">
+      <c r="H40" s="2" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41" s="1" t="s">
+    <row r="41" spans="1:8" ht="70" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B41" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C41" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="D41" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="E41" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="F41" s="2">
-        <v>46249</v>
-      </c>
-      <c r="G41" s="1" t="s">
+      <c r="F41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G41" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="H41" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42" s="1" t="s">
+    <row r="42" spans="1:8" ht="70" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="D42" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="E42" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="F42" s="2">
-        <v>46249</v>
-      </c>
-      <c r="G42" s="1" t="s">
+      <c r="F42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G42" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H42" s="1" t="s">
+      <c r="H42" s="2" t="s">
         <v>263</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="98" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="H43" s="2"/>
+    </row>
+    <row r="44" spans="1:8" ht="112" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="H44" s="2"/>
+    </row>
+    <row r="45" spans="1:8" ht="98" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="H45" s="2"/>
+    </row>
+    <row r="46" spans="1:8" ht="84" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="98" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="98" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="H48" s="2"/>
+    </row>
+    <row r="49" spans="1:8" ht="98" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="H49" s="2"/>
+    </row>
+    <row r="50" spans="1:8" ht="112" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="84" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="112" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="140" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" ht="154" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="140" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" ht="140" x14ac:dyDescent="0.2">
+      <c r="A56" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="H56" s="2"/>
+    </row>
+    <row r="57" spans="1:8" ht="126" x14ac:dyDescent="0.2">
+      <c r="A57" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="H57" s="2"/>
+    </row>
+    <row r="58" spans="1:8" ht="126" x14ac:dyDescent="0.2">
+      <c r="A58" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" ht="140" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" ht="98" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" ht="140" x14ac:dyDescent="0.2">
+      <c r="A61" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>385</v>
       </c>
     </row>
   </sheetData>

</xml_diff>